<commit_message>
FSEL-8531: fix report pt
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/ReportPTEventDistrictSchool.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/ReportPTEventDistrictSchool.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\multiple-subject\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BE5866F-BCA5-4510-9CEE-5E7C7B9453C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{77EED0B8-1FC3-456B-8AF6-DD57EB641DA1}"/>
+    <workbookView xWindow="-28920" yWindow="-135" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="152511" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
   <si>
     <t>TEMPLATE BÁO CÁO SỰ KIỆN SỞ HN</t>
   </si>
@@ -58,27 +57,6 @@
   </si>
   <si>
     <t>(Thể hiện năng lực của học viên sẵn sàng bắt đầu khóa học)</t>
-  </si>
-  <si>
-    <t>A1</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
-    <t>A2</t>
-  </si>
-  <si>
-    <t>B1</t>
-  </si>
-  <si>
-    <t>B1+</t>
-  </si>
-  <si>
-    <t>B2</t>
-  </si>
-  <si>
-    <t>C1</t>
   </si>
   <si>
     <t>Trường</t>
@@ -102,12 +80,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -115,27 +93,27 @@
       <b/>
       <sz val="14"/>
       <color rgb="FFC00000"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -143,7 +121,7 @@
       <i/>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -167,7 +145,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -285,39 +263,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -328,59 +278,47 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -695,11 +633,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16CA2A96-CFCD-46BA-B64D-76D2E518123B}">
-  <dimension ref="A1:W8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:W7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:23" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -726,7 +664,7 @@
       <c r="V1" s="2"/>
       <c r="W1" s="2"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -803,178 +741,129 @@
       <c r="V4" s="4"/>
       <c r="W4" s="4"/>
     </row>
-    <row r="5" spans="1:23" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
-      <c r="M5" s="7"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7"/>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="7"/>
-      <c r="R5" s="7"/>
-      <c r="S5" s="7"/>
-      <c r="T5" s="7"/>
-      <c r="U5" s="7"/>
-      <c r="V5" s="7"/>
-      <c r="W5" s="7"/>
+    <row r="5" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
+      <c r="P5" s="13"/>
+      <c r="Q5" s="13"/>
+      <c r="R5" s="13"/>
+      <c r="S5" s="13"/>
+      <c r="T5" s="13"/>
+      <c r="U5" s="13"/>
+      <c r="V5" s="13"/>
+      <c r="W5" s="13"/>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="9" t="s">
+      <c r="B6" s="8"/>
+      <c r="C6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="I6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="J6" s="9" t="s">
+      <c r="J6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="K6" s="9" t="s">
+      <c r="K6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="L6" s="10" t="s">
+      <c r="L6" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="11"/>
-      <c r="S6" s="11"/>
-      <c r="T6" s="11"/>
-      <c r="U6" s="11"/>
-      <c r="V6" s="11"/>
-      <c r="W6" s="12"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
+      <c r="R6" s="15"/>
+      <c r="S6" s="15"/>
+      <c r="T6" s="15"/>
+      <c r="U6" s="15"/>
+      <c r="V6" s="15"/>
+      <c r="W6" s="16"/>
     </row>
-    <row r="7" spans="1:23" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A7" s="13"/>
-      <c r="B7" s="22" t="s">
+    <row r="7" spans="1:23" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="11"/>
+      <c r="B7" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="13"/>
-      <c r="D7" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" s="14" t="s">
+      <c r="C7" s="11"/>
+      <c r="D7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="I7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="14" t="s">
+      <c r="J7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K7" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="L7" s="15" t="s">
+      <c r="K7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="L7" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="M7" s="16"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="16"/>
-      <c r="Q7" s="16"/>
-      <c r="R7" s="16"/>
-      <c r="S7" s="16"/>
-      <c r="T7" s="16"/>
-      <c r="U7" s="16"/>
-      <c r="V7" s="16"/>
-      <c r="W7" s="17"/>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A8" s="18"/>
-      <c r="B8" s="23"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="M8" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="N8" s="20" t="s">
-        <v>13</v>
-      </c>
-      <c r="O8" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="P8" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q8" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="R8" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="S8" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="T8" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="U8" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="V8" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="W8" s="20" t="s">
-        <v>12</v>
-      </c>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="18"/>
+      <c r="Q7" s="18"/>
+      <c r="R7" s="18"/>
+      <c r="S7" s="18"/>
+      <c r="T7" s="18"/>
+      <c r="U7" s="18"/>
+      <c r="V7" s="18"/>
+      <c r="W7" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="C6:C7"/>
     <mergeCell ref="A5:W5"/>
     <mergeCell ref="L6:W6"/>
     <mergeCell ref="L7:W7"/>

</xml_diff>